<commit_message>
fix: add persistent local user storage fallback to registration and login when remote DB is offline
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -497,7 +497,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>04-09-2026 22:00:55</v>
+        <v>04-09-2026 22:19:16</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -505,28 +505,28 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B3" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C3" t="str">
         <v>7th</v>
       </c>
       <c r="D3" t="str">
-        <v>Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E3" t="str">
-        <v>Chapter 1: Measurement &amp; Motion</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F3" t="str">
-        <v>Interactive Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G3">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H3" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I3">
         <v>10</v>
@@ -538,10 +538,10 @@
         <v>1</v>
       </c>
       <c r="L3" t="str">
-        <v>05:30 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M3" t="str">
-        <v>04-09-2026 14:15:22</v>
+        <v>04-09-2026 22:00:55</v>
       </c>
       <c r="N3" t="str">
         <v>PASSED</v>
@@ -558,34 +558,34 @@
         <v>7th</v>
       </c>
       <c r="D4" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E4" t="str">
-        <v>Chapter 1: Number System: Integers</v>
+        <v>Chapter 1: Measurement &amp; Motion</v>
       </c>
       <c r="F4" t="str">
-        <v>Integer Operations Challenge</v>
+        <v>Interactive Chapter Quiz</v>
       </c>
       <c r="G4">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H4" t="str">
-        <v>80%</v>
+        <v>90%</v>
       </c>
       <c r="I4">
         <v>10</v>
       </c>
       <c r="J4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L4" t="str">
-        <v>06:15 mins</v>
+        <v>05:30 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>04-09-2026 15:10:05</v>
+        <v>04-09-2026 14:15:22</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -602,34 +602,34 @@
         <v>7th</v>
       </c>
       <c r="D5" t="str">
-        <v>English</v>
+        <v>Mathematics</v>
       </c>
       <c r="E5" t="str">
-        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
+        <v>Chapter 1: Number System: Integers</v>
       </c>
       <c r="F5" t="str">
-        <v>Grammar &amp; Vocabulary Quiz</v>
+        <v>Integer Operations Challenge</v>
       </c>
       <c r="G5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H5" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I5">
         <v>10</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L5" t="str">
-        <v>04:40 mins</v>
+        <v>06:15 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>04-09-2026 15:45:18</v>
+        <v>04-09-2026 15:10:05</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -637,22 +637,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B6" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C6" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D6" t="str">
-        <v>Tamil</v>
+        <v>English</v>
       </c>
       <c r="E6" t="str">
-        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
+        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
       </c>
       <c r="F6" t="str">
-        <v>Tamil Literature Quiz</v>
+        <v>Grammar &amp; Vocabulary Quiz</v>
       </c>
       <c r="G6">
         <v>100</v>
@@ -670,10 +670,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="str">
-        <v>04:15 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>04-09-2026 11:20:45</v>
+        <v>04-09-2026 15:45:18</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -690,34 +690,34 @@
         <v>8th</v>
       </c>
       <c r="D7" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E7" t="str">
-        <v>Chapter 1: Measurement</v>
+        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
       </c>
       <c r="F7" t="str">
-        <v>SI Unit &amp; Mechanics Quiz</v>
+        <v>Tamil Literature Quiz</v>
       </c>
       <c r="G7">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H7" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I7">
         <v>10</v>
       </c>
       <c r="J7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" t="str">
-        <v>05:05 mins</v>
+        <v>04:15 mins</v>
       </c>
       <c r="M7" t="str">
-        <v>04-09-2026 12:35:10</v>
+        <v>04-09-2026 11:20:45</v>
       </c>
       <c r="N7" t="str">
         <v>PASSED</v>
@@ -725,43 +725,43 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B8" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C8" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D8" t="str">
         <v>Science</v>
       </c>
       <c r="E8" t="str">
-        <v>Chapter 1: Measurements &amp; Motion</v>
+        <v>Chapter 1: Measurement</v>
       </c>
       <c r="F8" t="str">
-        <v>Motion &amp; Scales Quest</v>
+        <v>SI Unit &amp; Mechanics Quiz</v>
       </c>
       <c r="G8">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H8" t="str">
-        <v>70%</v>
+        <v>90%</v>
       </c>
       <c r="I8">
         <v>10</v>
       </c>
       <c r="J8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L8" t="str">
-        <v>07:20 mins</v>
+        <v>05:05 mins</v>
       </c>
       <c r="M8" t="str">
-        <v>04-09-2026 09:30:12</v>
+        <v>04-09-2026 12:35:10</v>
       </c>
       <c r="N8" t="str">
         <v>PASSED</v>
@@ -778,37 +778,37 @@
         <v>6th</v>
       </c>
       <c r="D9" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E9" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurements &amp; Motion</v>
       </c>
       <c r="F9" t="str">
-        <v>Numbers Mastery Quiz</v>
+        <v>Motion &amp; Scales Quest</v>
       </c>
       <c r="G9">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H9" t="str">
-        <v>60%</v>
+        <v>70%</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" t="str">
-        <v>08:15 mins</v>
+        <v>07:20 mins</v>
       </c>
       <c r="M9" t="str">
-        <v>04-09-2026 10:15:30</v>
+        <v>04-09-2026 09:30:12</v>
       </c>
       <c r="N9" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
     </row>
     <row r="10">
@@ -828,72 +828,72 @@
         <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F10" t="str">
-        <v>Numbers Mastery Quiz (Retry)</v>
+        <v>Numbers Mastery Quiz</v>
       </c>
       <c r="G10">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="H10" t="str">
-        <v>90%</v>
+        <v>60%</v>
       </c>
       <c r="I10">
         <v>10</v>
       </c>
       <c r="J10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L10" t="str">
-        <v>05:45 mins</v>
+        <v>08:15 mins</v>
       </c>
       <c r="M10" t="str">
-        <v>04-09-2026 10:45:00</v>
+        <v>04-09-2026 10:15:30</v>
       </c>
       <c r="N10" t="str">
-        <v>PASSED</v>
+        <v>FAILED</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Divya Nair</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B11" t="str">
-        <v>USER004</v>
+        <v>USER003</v>
       </c>
       <c r="C11" t="str">
-        <v>5th</v>
+        <v>6th</v>
       </c>
       <c r="D11" t="str">
-        <v>Social Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E11" t="str">
-        <v>Chapter 1: Introduction to Social Science</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F11" t="str">
-        <v>Continents &amp; Oceans Quiz</v>
+        <v>Numbers Mastery Quiz (Retry)</v>
       </c>
       <c r="G11">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H11" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I11">
         <v>10</v>
       </c>
       <c r="J11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="str">
-        <v>03:50 mins</v>
+        <v>05:45 mins</v>
       </c>
       <c r="M11" t="str">
-        <v>04-09-2026 13:00:25</v>
+        <v>04-09-2026 10:45:00</v>
       </c>
       <c r="N11" t="str">
         <v>PASSED</v>
@@ -901,22 +901,22 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Student Scholar</v>
+        <v>Divya Nair</v>
       </c>
       <c r="B12" t="str">
-        <v>usr-student-1</v>
+        <v>USER004</v>
       </c>
       <c r="C12" t="str">
-        <v>4th</v>
+        <v>5th</v>
       </c>
       <c r="D12" t="str">
-        <v>Tamil</v>
+        <v>Social Science</v>
       </c>
       <c r="E12" t="str">
-        <v>Chapter 1: அன்னைத் தமிழே</v>
+        <v>Chapter 1: Introduction to Social Science</v>
       </c>
       <c r="F12" t="str">
-        <v>Tamil Poem &amp; Grammar Quiz</v>
+        <v>Continents &amp; Oceans Quiz</v>
       </c>
       <c r="G12">
         <v>100</v>
@@ -934,10 +934,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="str">
-        <v>04:10 mins</v>
+        <v>03:50 mins</v>
       </c>
       <c r="M12" t="str">
-        <v>04-09-2026 14:00:15</v>
+        <v>04-09-2026 13:00:25</v>
       </c>
       <c r="N12" t="str">
         <v>PASSED</v>
@@ -951,45 +951,89 @@
         <v>usr-student-1</v>
       </c>
       <c r="C13" t="str">
-        <v>11th</v>
+        <v>4th</v>
       </c>
       <c r="D13" t="str">
-        <v>Chemistry</v>
+        <v>Tamil</v>
       </c>
       <c r="E13" t="str">
-        <v>Chapter 3: Periodic Classification</v>
+        <v>Chapter 1: அன்னைத் தமிழே</v>
       </c>
       <c r="F13" t="str">
-        <v>Grid Reconstruction Game</v>
+        <v>Tamil Poem &amp; Grammar Quiz</v>
       </c>
       <c r="G13">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="H13" t="str">
         <v>100%</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13" t="str">
+        <v>04:10 mins</v>
+      </c>
+      <c r="M13" t="str">
+        <v>04-09-2026 14:00:15</v>
+      </c>
+      <c r="N13" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B14" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C14" t="str">
+        <v>11th</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Chapter 3: Periodic Classification</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Grid Reconstruction Game</v>
+      </c>
+      <c r="G14">
+        <v>150</v>
+      </c>
+      <c r="H14" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I14">
+        <v>3</v>
+      </c>
+      <c r="J14">
+        <v>3</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" t="str">
         <v>03:20 mins</v>
       </c>
-      <c r="M13" t="str">
+      <c r="M14" t="str">
         <v>04-09-2026 15:30:00</v>
       </c>
-      <c r="N13" t="str">
+      <c r="N14" t="str">
         <v>COMPLETED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): complete theme overhaul inspired by modern educational quiz design
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -497,7 +497,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>04-09-2026 22:19:16</v>
+        <v>04-09-2026 23:01:42</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -541,7 +541,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M3" t="str">
-        <v>04-09-2026 22:00:55</v>
+        <v>04-09-2026 22:19:16</v>
       </c>
       <c r="N3" t="str">
         <v>PASSED</v>
@@ -549,28 +549,28 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B4" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C4" t="str">
         <v>7th</v>
       </c>
       <c r="D4" t="str">
-        <v>Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E4" t="str">
-        <v>Chapter 1: Measurement &amp; Motion</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F4" t="str">
-        <v>Interactive Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G4">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H4" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -582,10 +582,10 @@
         <v>1</v>
       </c>
       <c r="L4" t="str">
-        <v>05:30 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>04-09-2026 14:15:22</v>
+        <v>04-09-2026 22:00:55</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -602,34 +602,34 @@
         <v>7th</v>
       </c>
       <c r="D5" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E5" t="str">
-        <v>Chapter 1: Number System: Integers</v>
+        <v>Chapter 1: Measurement &amp; Motion</v>
       </c>
       <c r="F5" t="str">
-        <v>Integer Operations Challenge</v>
+        <v>Interactive Chapter Quiz</v>
       </c>
       <c r="G5">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H5" t="str">
-        <v>80%</v>
+        <v>90%</v>
       </c>
       <c r="I5">
         <v>10</v>
       </c>
       <c r="J5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L5" t="str">
-        <v>06:15 mins</v>
+        <v>05:30 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>04-09-2026 15:10:05</v>
+        <v>04-09-2026 14:15:22</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -646,34 +646,34 @@
         <v>7th</v>
       </c>
       <c r="D6" t="str">
-        <v>English</v>
+        <v>Mathematics</v>
       </c>
       <c r="E6" t="str">
-        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
+        <v>Chapter 1: Number System: Integers</v>
       </c>
       <c r="F6" t="str">
-        <v>Grammar &amp; Vocabulary Quiz</v>
+        <v>Integer Operations Challenge</v>
       </c>
       <c r="G6">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H6" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I6">
         <v>10</v>
       </c>
       <c r="J6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L6" t="str">
-        <v>04:40 mins</v>
+        <v>06:15 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>04-09-2026 15:45:18</v>
+        <v>04-09-2026 15:10:05</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -681,22 +681,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B7" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C7" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D7" t="str">
-        <v>Tamil</v>
+        <v>English</v>
       </c>
       <c r="E7" t="str">
-        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
+        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
       </c>
       <c r="F7" t="str">
-        <v>Tamil Literature Quiz</v>
+        <v>Grammar &amp; Vocabulary Quiz</v>
       </c>
       <c r="G7">
         <v>100</v>
@@ -714,10 +714,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="str">
-        <v>04:15 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M7" t="str">
-        <v>04-09-2026 11:20:45</v>
+        <v>04-09-2026 15:45:18</v>
       </c>
       <c r="N7" t="str">
         <v>PASSED</v>
@@ -734,34 +734,34 @@
         <v>8th</v>
       </c>
       <c r="D8" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E8" t="str">
-        <v>Chapter 1: Measurement</v>
+        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
       </c>
       <c r="F8" t="str">
-        <v>SI Unit &amp; Mechanics Quiz</v>
+        <v>Tamil Literature Quiz</v>
       </c>
       <c r="G8">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H8" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I8">
         <v>10</v>
       </c>
       <c r="J8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" t="str">
-        <v>05:05 mins</v>
+        <v>04:15 mins</v>
       </c>
       <c r="M8" t="str">
-        <v>04-09-2026 12:35:10</v>
+        <v>04-09-2026 11:20:45</v>
       </c>
       <c r="N8" t="str">
         <v>PASSED</v>
@@ -769,43 +769,43 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B9" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C9" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D9" t="str">
         <v>Science</v>
       </c>
       <c r="E9" t="str">
-        <v>Chapter 1: Measurements &amp; Motion</v>
+        <v>Chapter 1: Measurement</v>
       </c>
       <c r="F9" t="str">
-        <v>Motion &amp; Scales Quest</v>
+        <v>SI Unit &amp; Mechanics Quiz</v>
       </c>
       <c r="G9">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H9" t="str">
-        <v>70%</v>
+        <v>90%</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" t="str">
-        <v>07:20 mins</v>
+        <v>05:05 mins</v>
       </c>
       <c r="M9" t="str">
-        <v>04-09-2026 09:30:12</v>
+        <v>04-09-2026 12:35:10</v>
       </c>
       <c r="N9" t="str">
         <v>PASSED</v>
@@ -822,37 +822,37 @@
         <v>6th</v>
       </c>
       <c r="D10" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E10" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurements &amp; Motion</v>
       </c>
       <c r="F10" t="str">
-        <v>Numbers Mastery Quiz</v>
+        <v>Motion &amp; Scales Quest</v>
       </c>
       <c r="G10">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H10" t="str">
-        <v>60%</v>
+        <v>70%</v>
       </c>
       <c r="I10">
         <v>10</v>
       </c>
       <c r="J10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" t="str">
-        <v>08:15 mins</v>
+        <v>07:20 mins</v>
       </c>
       <c r="M10" t="str">
-        <v>04-09-2026 10:15:30</v>
+        <v>04-09-2026 09:30:12</v>
       </c>
       <c r="N10" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
     </row>
     <row r="11">
@@ -872,72 +872,72 @@
         <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F11" t="str">
-        <v>Numbers Mastery Quiz (Retry)</v>
+        <v>Numbers Mastery Quiz</v>
       </c>
       <c r="G11">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="H11" t="str">
-        <v>90%</v>
+        <v>60%</v>
       </c>
       <c r="I11">
         <v>10</v>
       </c>
       <c r="J11">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L11" t="str">
-        <v>05:45 mins</v>
+        <v>08:15 mins</v>
       </c>
       <c r="M11" t="str">
-        <v>04-09-2026 10:45:00</v>
+        <v>04-09-2026 10:15:30</v>
       </c>
       <c r="N11" t="str">
-        <v>PASSED</v>
+        <v>FAILED</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Divya Nair</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B12" t="str">
-        <v>USER004</v>
+        <v>USER003</v>
       </c>
       <c r="C12" t="str">
-        <v>5th</v>
+        <v>6th</v>
       </c>
       <c r="D12" t="str">
-        <v>Social Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E12" t="str">
-        <v>Chapter 1: Introduction to Social Science</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F12" t="str">
-        <v>Continents &amp; Oceans Quiz</v>
+        <v>Numbers Mastery Quiz (Retry)</v>
       </c>
       <c r="G12">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H12" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I12">
         <v>10</v>
       </c>
       <c r="J12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="str">
-        <v>03:50 mins</v>
+        <v>05:45 mins</v>
       </c>
       <c r="M12" t="str">
-        <v>04-09-2026 13:00:25</v>
+        <v>04-09-2026 10:45:00</v>
       </c>
       <c r="N12" t="str">
         <v>PASSED</v>
@@ -945,22 +945,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Student Scholar</v>
+        <v>Divya Nair</v>
       </c>
       <c r="B13" t="str">
-        <v>usr-student-1</v>
+        <v>USER004</v>
       </c>
       <c r="C13" t="str">
-        <v>4th</v>
+        <v>5th</v>
       </c>
       <c r="D13" t="str">
-        <v>Tamil</v>
+        <v>Social Science</v>
       </c>
       <c r="E13" t="str">
-        <v>Chapter 1: அன்னைத் தமிழே</v>
+        <v>Chapter 1: Introduction to Social Science</v>
       </c>
       <c r="F13" t="str">
-        <v>Tamil Poem &amp; Grammar Quiz</v>
+        <v>Continents &amp; Oceans Quiz</v>
       </c>
       <c r="G13">
         <v>100</v>
@@ -978,10 +978,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="str">
-        <v>04:10 mins</v>
+        <v>03:50 mins</v>
       </c>
       <c r="M13" t="str">
-        <v>04-09-2026 14:00:15</v>
+        <v>04-09-2026 13:00:25</v>
       </c>
       <c r="N13" t="str">
         <v>PASSED</v>
@@ -995,45 +995,89 @@
         <v>usr-student-1</v>
       </c>
       <c r="C14" t="str">
-        <v>11th</v>
+        <v>4th</v>
       </c>
       <c r="D14" t="str">
-        <v>Chemistry</v>
+        <v>Tamil</v>
       </c>
       <c r="E14" t="str">
-        <v>Chapter 3: Periodic Classification</v>
+        <v>Chapter 1: அன்னைத் தமிழே</v>
       </c>
       <c r="F14" t="str">
-        <v>Grid Reconstruction Game</v>
+        <v>Tamil Poem &amp; Grammar Quiz</v>
       </c>
       <c r="G14">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="H14" t="str">
         <v>100%</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14" t="str">
+        <v>04:10 mins</v>
+      </c>
+      <c r="M14" t="str">
+        <v>04-09-2026 14:00:15</v>
+      </c>
+      <c r="N14" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B15" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C15" t="str">
+        <v>11th</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Chapter 3: Periodic Classification</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Grid Reconstruction Game</v>
+      </c>
+      <c r="G15">
+        <v>150</v>
+      </c>
+      <c r="H15" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15" t="str">
         <v>03:20 mins</v>
       </c>
-      <c r="M14" t="str">
+      <c r="M15" t="str">
         <v>04-09-2026 15:30:00</v>
       </c>
-      <c r="N14" t="str">
+      <c r="N15" t="str">
         <v>COMPLETED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): resolve light mode text visibility in sidebar navigation and charts
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -497,7 +497,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>04-09-2026 23:01:42</v>
+        <v>04-09-2026 23:14:28</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -541,7 +541,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M3" t="str">
-        <v>04-09-2026 22:19:16</v>
+        <v>04-09-2026 23:01:42</v>
       </c>
       <c r="N3" t="str">
         <v>PASSED</v>
@@ -585,7 +585,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>04-09-2026 22:00:55</v>
+        <v>04-09-2026 22:19:16</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -593,28 +593,28 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B5" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C5" t="str">
         <v>7th</v>
       </c>
       <c r="D5" t="str">
-        <v>Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E5" t="str">
-        <v>Chapter 1: Measurement &amp; Motion</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F5" t="str">
-        <v>Interactive Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G5">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H5" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I5">
         <v>10</v>
@@ -626,10 +626,10 @@
         <v>1</v>
       </c>
       <c r="L5" t="str">
-        <v>05:30 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>04-09-2026 14:15:22</v>
+        <v>04-09-2026 22:00:55</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -646,34 +646,34 @@
         <v>7th</v>
       </c>
       <c r="D6" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E6" t="str">
-        <v>Chapter 1: Number System: Integers</v>
+        <v>Chapter 1: Measurement &amp; Motion</v>
       </c>
       <c r="F6" t="str">
-        <v>Integer Operations Challenge</v>
+        <v>Interactive Chapter Quiz</v>
       </c>
       <c r="G6">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H6" t="str">
-        <v>80%</v>
+        <v>90%</v>
       </c>
       <c r="I6">
         <v>10</v>
       </c>
       <c r="J6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" t="str">
-        <v>06:15 mins</v>
+        <v>05:30 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>04-09-2026 15:10:05</v>
+        <v>04-09-2026 14:15:22</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -690,34 +690,34 @@
         <v>7th</v>
       </c>
       <c r="D7" t="str">
-        <v>English</v>
+        <v>Mathematics</v>
       </c>
       <c r="E7" t="str">
-        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
+        <v>Chapter 1: Number System: Integers</v>
       </c>
       <c r="F7" t="str">
-        <v>Grammar &amp; Vocabulary Quiz</v>
+        <v>Integer Operations Challenge</v>
       </c>
       <c r="G7">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H7" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I7">
         <v>10</v>
       </c>
       <c r="J7">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L7" t="str">
-        <v>04:40 mins</v>
+        <v>06:15 mins</v>
       </c>
       <c r="M7" t="str">
-        <v>04-09-2026 15:45:18</v>
+        <v>04-09-2026 15:10:05</v>
       </c>
       <c r="N7" t="str">
         <v>PASSED</v>
@@ -725,22 +725,22 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B8" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C8" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D8" t="str">
-        <v>Tamil</v>
+        <v>English</v>
       </c>
       <c r="E8" t="str">
-        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
+        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
       </c>
       <c r="F8" t="str">
-        <v>Tamil Literature Quiz</v>
+        <v>Grammar &amp; Vocabulary Quiz</v>
       </c>
       <c r="G8">
         <v>100</v>
@@ -758,10 +758,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="str">
-        <v>04:15 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M8" t="str">
-        <v>04-09-2026 11:20:45</v>
+        <v>04-09-2026 15:45:18</v>
       </c>
       <c r="N8" t="str">
         <v>PASSED</v>
@@ -778,34 +778,34 @@
         <v>8th</v>
       </c>
       <c r="D9" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E9" t="str">
-        <v>Chapter 1: Measurement</v>
+        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
       </c>
       <c r="F9" t="str">
-        <v>SI Unit &amp; Mechanics Quiz</v>
+        <v>Tamil Literature Quiz</v>
       </c>
       <c r="G9">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H9" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="str">
-        <v>05:05 mins</v>
+        <v>04:15 mins</v>
       </c>
       <c r="M9" t="str">
-        <v>04-09-2026 12:35:10</v>
+        <v>04-09-2026 11:20:45</v>
       </c>
       <c r="N9" t="str">
         <v>PASSED</v>
@@ -813,43 +813,43 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B10" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C10" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D10" t="str">
         <v>Science</v>
       </c>
       <c r="E10" t="str">
-        <v>Chapter 1: Measurements &amp; Motion</v>
+        <v>Chapter 1: Measurement</v>
       </c>
       <c r="F10" t="str">
-        <v>Motion &amp; Scales Quest</v>
+        <v>SI Unit &amp; Mechanics Quiz</v>
       </c>
       <c r="G10">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H10" t="str">
-        <v>70%</v>
+        <v>90%</v>
       </c>
       <c r="I10">
         <v>10</v>
       </c>
       <c r="J10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" t="str">
-        <v>07:20 mins</v>
+        <v>05:05 mins</v>
       </c>
       <c r="M10" t="str">
-        <v>04-09-2026 09:30:12</v>
+        <v>04-09-2026 12:35:10</v>
       </c>
       <c r="N10" t="str">
         <v>PASSED</v>
@@ -866,37 +866,37 @@
         <v>6th</v>
       </c>
       <c r="D11" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E11" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurements &amp; Motion</v>
       </c>
       <c r="F11" t="str">
-        <v>Numbers Mastery Quiz</v>
+        <v>Motion &amp; Scales Quest</v>
       </c>
       <c r="G11">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H11" t="str">
-        <v>60%</v>
+        <v>70%</v>
       </c>
       <c r="I11">
         <v>10</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L11" t="str">
-        <v>08:15 mins</v>
+        <v>07:20 mins</v>
       </c>
       <c r="M11" t="str">
-        <v>04-09-2026 10:15:30</v>
+        <v>04-09-2026 09:30:12</v>
       </c>
       <c r="N11" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
     </row>
     <row r="12">
@@ -916,72 +916,72 @@
         <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F12" t="str">
-        <v>Numbers Mastery Quiz (Retry)</v>
+        <v>Numbers Mastery Quiz</v>
       </c>
       <c r="G12">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="H12" t="str">
-        <v>90%</v>
+        <v>60%</v>
       </c>
       <c r="I12">
         <v>10</v>
       </c>
       <c r="J12">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L12" t="str">
-        <v>05:45 mins</v>
+        <v>08:15 mins</v>
       </c>
       <c r="M12" t="str">
-        <v>04-09-2026 10:45:00</v>
+        <v>04-09-2026 10:15:30</v>
       </c>
       <c r="N12" t="str">
-        <v>PASSED</v>
+        <v>FAILED</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Divya Nair</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B13" t="str">
-        <v>USER004</v>
+        <v>USER003</v>
       </c>
       <c r="C13" t="str">
-        <v>5th</v>
+        <v>6th</v>
       </c>
       <c r="D13" t="str">
-        <v>Social Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E13" t="str">
-        <v>Chapter 1: Introduction to Social Science</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F13" t="str">
-        <v>Continents &amp; Oceans Quiz</v>
+        <v>Numbers Mastery Quiz (Retry)</v>
       </c>
       <c r="G13">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H13" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I13">
         <v>10</v>
       </c>
       <c r="J13">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" t="str">
-        <v>03:50 mins</v>
+        <v>05:45 mins</v>
       </c>
       <c r="M13" t="str">
-        <v>04-09-2026 13:00:25</v>
+        <v>04-09-2026 10:45:00</v>
       </c>
       <c r="N13" t="str">
         <v>PASSED</v>
@@ -989,22 +989,22 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Student Scholar</v>
+        <v>Divya Nair</v>
       </c>
       <c r="B14" t="str">
-        <v>usr-student-1</v>
+        <v>USER004</v>
       </c>
       <c r="C14" t="str">
-        <v>4th</v>
+        <v>5th</v>
       </c>
       <c r="D14" t="str">
-        <v>Tamil</v>
+        <v>Social Science</v>
       </c>
       <c r="E14" t="str">
-        <v>Chapter 1: அன்னைத் தமிழே</v>
+        <v>Chapter 1: Introduction to Social Science</v>
       </c>
       <c r="F14" t="str">
-        <v>Tamil Poem &amp; Grammar Quiz</v>
+        <v>Continents &amp; Oceans Quiz</v>
       </c>
       <c r="G14">
         <v>100</v>
@@ -1022,10 +1022,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="str">
-        <v>04:10 mins</v>
+        <v>03:50 mins</v>
       </c>
       <c r="M14" t="str">
-        <v>04-09-2026 14:00:15</v>
+        <v>04-09-2026 13:00:25</v>
       </c>
       <c r="N14" t="str">
         <v>PASSED</v>
@@ -1039,45 +1039,89 @@
         <v>usr-student-1</v>
       </c>
       <c r="C15" t="str">
-        <v>11th</v>
+        <v>4th</v>
       </c>
       <c r="D15" t="str">
-        <v>Chemistry</v>
+        <v>Tamil</v>
       </c>
       <c r="E15" t="str">
-        <v>Chapter 3: Periodic Classification</v>
+        <v>Chapter 1: அன்னைத் தமிழே</v>
       </c>
       <c r="F15" t="str">
-        <v>Grid Reconstruction Game</v>
+        <v>Tamil Poem &amp; Grammar Quiz</v>
       </c>
       <c r="G15">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="H15" t="str">
         <v>100%</v>
       </c>
       <c r="I15">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15" t="str">
+        <v>04:10 mins</v>
+      </c>
+      <c r="M15" t="str">
+        <v>04-09-2026 14:00:15</v>
+      </c>
+      <c r="N15" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B16" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C16" t="str">
+        <v>11th</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Chapter 3: Periodic Classification</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Grid Reconstruction Game</v>
+      </c>
+      <c r="G16">
+        <v>150</v>
+      </c>
+      <c r="H16" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16" t="str">
         <v>03:20 mins</v>
       </c>
-      <c r="M15" t="str">
+      <c r="M16" t="str">
         <v>04-09-2026 15:30:00</v>
       </c>
-      <c r="N15" t="str">
+      <c r="N16" t="str">
         <v>COMPLETED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reports): sync latest user activity history records and generated Excel report
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N18"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -461,28 +461,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Priya Sharma</v>
+        <v>Student Scholar</v>
       </c>
       <c r="B2" t="str">
-        <v>USER002</v>
+        <v>user-student-1</v>
       </c>
       <c r="C2" t="str">
-        <v>7th</v>
+        <v>4th</v>
       </c>
       <c r="D2" t="str">
-        <v>Mathematics</v>
+        <v>Tamil</v>
       </c>
       <c r="E2" t="str">
-        <v>Chapter 2: Algebra Expressions</v>
+        <v>அன்னைத் தமிழே</v>
       </c>
       <c r="F2" t="str">
-        <v>Algebra Mastery Quiz</v>
+        <v>Tamil Chapter Quiz</v>
       </c>
       <c r="G2">
-        <v>95</v>
+        <v>900</v>
       </c>
       <c r="H2" t="str">
-        <v>95%</v>
+        <v>90%</v>
       </c>
       <c r="I2">
         <v>10</v>
@@ -494,10 +494,10 @@
         <v>1</v>
       </c>
       <c r="L2" t="str">
-        <v>04:40 mins</v>
+        <v>02:21 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>04-09-2026 23:14:28</v>
+        <v>05-09-2026 10:54:56</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -505,28 +505,28 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Priya Sharma</v>
+        <v>Student Scholar</v>
       </c>
       <c r="B3" t="str">
-        <v>USER002</v>
+        <v>user-student-1</v>
       </c>
       <c r="C3" t="str">
         <v>7th</v>
       </c>
       <c r="D3" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E3" t="str">
-        <v>Chapter 2: Algebra Expressions</v>
+        <v>ch-tam4-1</v>
       </c>
       <c r="F3" t="str">
-        <v>Algebra Mastery Quiz</v>
+        <v>அன்னைத் தமிழ் அரங்கம்</v>
       </c>
       <c r="G3">
-        <v>95</v>
+        <v>900</v>
       </c>
       <c r="H3" t="str">
-        <v>95%</v>
+        <v>90%</v>
       </c>
       <c r="I3">
         <v>10</v>
@@ -538,10 +538,10 @@
         <v>1</v>
       </c>
       <c r="L3" t="str">
-        <v>04:40 mins</v>
+        <v>02:21 mins</v>
       </c>
       <c r="M3" t="str">
-        <v>04-09-2026 23:01:42</v>
+        <v>05-09-2026 10:54:56</v>
       </c>
       <c r="N3" t="str">
         <v>PASSED</v>
@@ -585,7 +585,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>04-09-2026 22:19:16</v>
+        <v>04-09-2026 23:14:28</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -629,7 +629,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>04-09-2026 22:00:55</v>
+        <v>04-09-2026 23:01:42</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -637,28 +637,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B6" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C6" t="str">
         <v>7th</v>
       </c>
       <c r="D6" t="str">
-        <v>Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E6" t="str">
-        <v>Chapter 1: Measurement &amp; Motion</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F6" t="str">
-        <v>Interactive Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G6">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H6" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I6">
         <v>10</v>
@@ -670,10 +670,10 @@
         <v>1</v>
       </c>
       <c r="L6" t="str">
-        <v>05:30 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>04-09-2026 14:15:22</v>
+        <v>04-09-2026 22:19:16</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -681,10 +681,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B7" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C7" t="str">
         <v>7th</v>
@@ -693,31 +693,31 @@
         <v>Mathematics</v>
       </c>
       <c r="E7" t="str">
-        <v>Chapter 1: Number System: Integers</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F7" t="str">
-        <v>Integer Operations Challenge</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G7">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="H7" t="str">
-        <v>80%</v>
+        <v>95%</v>
       </c>
       <c r="I7">
         <v>10</v>
       </c>
       <c r="J7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" t="str">
-        <v>06:15 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M7" t="str">
-        <v>04-09-2026 15:10:05</v>
+        <v>04-09-2026 22:00:55</v>
       </c>
       <c r="N7" t="str">
         <v>PASSED</v>
@@ -734,34 +734,34 @@
         <v>7th</v>
       </c>
       <c r="D8" t="str">
-        <v>English</v>
+        <v>Science</v>
       </c>
       <c r="E8" t="str">
-        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
+        <v>Chapter 1: Measurement &amp; Motion</v>
       </c>
       <c r="F8" t="str">
-        <v>Grammar &amp; Vocabulary Quiz</v>
+        <v>Interactive Chapter Quiz</v>
       </c>
       <c r="G8">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H8" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I8">
         <v>10</v>
       </c>
       <c r="J8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="str">
-        <v>04:40 mins</v>
+        <v>05:30 mins</v>
       </c>
       <c r="M8" t="str">
-        <v>04-09-2026 15:45:18</v>
+        <v>04-09-2026 14:15:22</v>
       </c>
       <c r="N8" t="str">
         <v>PASSED</v>
@@ -769,43 +769,43 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B9" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C9" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D9" t="str">
-        <v>Tamil</v>
+        <v>Mathematics</v>
       </c>
       <c r="E9" t="str">
-        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
+        <v>Chapter 1: Number System: Integers</v>
       </c>
       <c r="F9" t="str">
-        <v>Tamil Literature Quiz</v>
+        <v>Integer Operations Challenge</v>
       </c>
       <c r="G9">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H9" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L9" t="str">
-        <v>04:15 mins</v>
+        <v>06:15 mins</v>
       </c>
       <c r="M9" t="str">
-        <v>04-09-2026 11:20:45</v>
+        <v>04-09-2026 15:10:05</v>
       </c>
       <c r="N9" t="str">
         <v>PASSED</v>
@@ -813,43 +813,43 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B10" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C10" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D10" t="str">
-        <v>Science</v>
+        <v>English</v>
       </c>
       <c r="E10" t="str">
-        <v>Chapter 1: Measurement</v>
+        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
       </c>
       <c r="F10" t="str">
-        <v>SI Unit &amp; Mechanics Quiz</v>
+        <v>Grammar &amp; Vocabulary Quiz</v>
       </c>
       <c r="G10">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H10" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I10">
         <v>10</v>
       </c>
       <c r="J10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="str">
-        <v>05:05 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M10" t="str">
-        <v>04-09-2026 12:35:10</v>
+        <v>04-09-2026 15:45:18</v>
       </c>
       <c r="N10" t="str">
         <v>PASSED</v>
@@ -857,43 +857,43 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B11" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C11" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D11" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E11" t="str">
-        <v>Chapter 1: Measurements &amp; Motion</v>
+        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
       </c>
       <c r="F11" t="str">
-        <v>Motion &amp; Scales Quest</v>
+        <v>Tamil Literature Quiz</v>
       </c>
       <c r="G11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="H11" t="str">
-        <v>70%</v>
+        <v>100%</v>
       </c>
       <c r="I11">
         <v>10</v>
       </c>
       <c r="J11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L11" t="str">
-        <v>07:20 mins</v>
+        <v>04:15 mins</v>
       </c>
       <c r="M11" t="str">
-        <v>04-09-2026 09:30:12</v>
+        <v>04-09-2026 11:20:45</v>
       </c>
       <c r="N11" t="str">
         <v>PASSED</v>
@@ -901,46 +901,46 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B12" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C12" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D12" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E12" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurement</v>
       </c>
       <c r="F12" t="str">
-        <v>Numbers Mastery Quiz</v>
+        <v>SI Unit &amp; Mechanics Quiz</v>
       </c>
       <c r="G12">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H12" t="str">
-        <v>60%</v>
+        <v>90%</v>
       </c>
       <c r="I12">
         <v>10</v>
       </c>
       <c r="J12">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" t="str">
-        <v>08:15 mins</v>
+        <v>05:05 mins</v>
       </c>
       <c r="M12" t="str">
-        <v>04-09-2026 10:15:30</v>
+        <v>04-09-2026 12:35:10</v>
       </c>
       <c r="N12" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
     </row>
     <row r="13">
@@ -954,34 +954,34 @@
         <v>6th</v>
       </c>
       <c r="D13" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E13" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurements &amp; Motion</v>
       </c>
       <c r="F13" t="str">
-        <v>Numbers Mastery Quiz (Retry)</v>
+        <v>Motion &amp; Scales Quest</v>
       </c>
       <c r="G13">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="H13" t="str">
-        <v>90%</v>
+        <v>70%</v>
       </c>
       <c r="I13">
         <v>10</v>
       </c>
       <c r="J13">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L13" t="str">
-        <v>05:45 mins</v>
+        <v>07:20 mins</v>
       </c>
       <c r="M13" t="str">
-        <v>04-09-2026 10:45:00</v>
+        <v>04-09-2026 09:30:12</v>
       </c>
       <c r="N13" t="str">
         <v>PASSED</v>
@@ -989,87 +989,87 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Divya Nair</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B14" t="str">
-        <v>USER004</v>
+        <v>USER003</v>
       </c>
       <c r="C14" t="str">
-        <v>5th</v>
+        <v>6th</v>
       </c>
       <c r="D14" t="str">
-        <v>Social Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E14" t="str">
-        <v>Chapter 1: Introduction to Social Science</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F14" t="str">
-        <v>Continents &amp; Oceans Quiz</v>
+        <v>Numbers Mastery Quiz</v>
       </c>
       <c r="G14">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="H14" t="str">
-        <v>100%</v>
+        <v>60%</v>
       </c>
       <c r="I14">
         <v>10</v>
       </c>
       <c r="J14">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L14" t="str">
-        <v>03:50 mins</v>
+        <v>08:15 mins</v>
       </c>
       <c r="M14" t="str">
-        <v>04-09-2026 13:00:25</v>
+        <v>04-09-2026 10:15:30</v>
       </c>
       <c r="N14" t="str">
-        <v>PASSED</v>
+        <v>FAILED</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Student Scholar</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B15" t="str">
-        <v>usr-student-1</v>
+        <v>USER003</v>
       </c>
       <c r="C15" t="str">
-        <v>4th</v>
+        <v>6th</v>
       </c>
       <c r="D15" t="str">
-        <v>Tamil</v>
+        <v>Mathematics</v>
       </c>
       <c r="E15" t="str">
-        <v>Chapter 1: அன்னைத் தமிழே</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F15" t="str">
-        <v>Tamil Poem &amp; Grammar Quiz</v>
+        <v>Numbers Mastery Quiz (Retry)</v>
       </c>
       <c r="G15">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H15" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I15">
         <v>10</v>
       </c>
       <c r="J15">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="str">
-        <v>04:10 mins</v>
+        <v>05:45 mins</v>
       </c>
       <c r="M15" t="str">
-        <v>04-09-2026 14:00:15</v>
+        <v>04-09-2026 10:45:00</v>
       </c>
       <c r="N15" t="str">
         <v>PASSED</v>
@@ -1077,51 +1077,139 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Student Scholar</v>
+        <v>Divya Nair</v>
       </c>
       <c r="B16" t="str">
-        <v>usr-student-1</v>
+        <v>USER004</v>
       </c>
       <c r="C16" t="str">
-        <v>11th</v>
+        <v>5th</v>
       </c>
       <c r="D16" t="str">
-        <v>Chemistry</v>
+        <v>Social Science</v>
       </c>
       <c r="E16" t="str">
-        <v>Chapter 3: Periodic Classification</v>
+        <v>Chapter 1: Introduction to Social Science</v>
       </c>
       <c r="F16" t="str">
-        <v>Grid Reconstruction Game</v>
+        <v>Continents &amp; Oceans Quiz</v>
       </c>
       <c r="G16">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="H16" t="str">
         <v>100%</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J16">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16" t="str">
+        <v>03:50 mins</v>
+      </c>
+      <c r="M16" t="str">
+        <v>04-09-2026 13:00:25</v>
+      </c>
+      <c r="N16" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B17" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C17" t="str">
+        <v>4th</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Tamil</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Chapter 1: அன்னைத் தமிழே</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Tamil Poem &amp; Grammar Quiz</v>
+      </c>
+      <c r="G17">
+        <v>100</v>
+      </c>
+      <c r="H17" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I17">
+        <v>10</v>
+      </c>
+      <c r="J17">
+        <v>10</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17" t="str">
+        <v>04:10 mins</v>
+      </c>
+      <c r="M17" t="str">
+        <v>04-09-2026 14:00:15</v>
+      </c>
+      <c r="N17" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B18" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C18" t="str">
+        <v>11th</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Chapter 3: Periodic Classification</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Grid Reconstruction Game</v>
+      </c>
+      <c r="G18">
+        <v>150</v>
+      </c>
+      <c r="H18" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I18">
+        <v>3</v>
+      </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18" t="str">
         <v>03:20 mins</v>
       </c>
-      <c r="M16" t="str">
+      <c r="M18" t="str">
         <v>04-09-2026 15:30:00</v>
       </c>
-      <c r="N16" t="str">
+      <c r="N18" t="str">
         <v>COMPLETED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(deployment): resolve 'No questions available' error with resilient curriculum fallback, CORS updates, and production URL handling
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -461,28 +461,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Student Scholar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B2" t="str">
-        <v>user-student-1</v>
+        <v>USER002</v>
       </c>
       <c r="C2" t="str">
-        <v>4th</v>
+        <v>7th</v>
       </c>
       <c r="D2" t="str">
-        <v>Tamil</v>
+        <v>Mathematics</v>
       </c>
       <c r="E2" t="str">
-        <v>அன்னைத் தமிழே</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F2" t="str">
-        <v>Tamil Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G2">
-        <v>900</v>
+        <v>95</v>
       </c>
       <c r="H2" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I2">
         <v>10</v>
@@ -494,10 +494,10 @@
         <v>1</v>
       </c>
       <c r="L2" t="str">
-        <v>02:21 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>05-09-2026 10:54:56</v>
+        <v>05-09-2026 12:37:53</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -511,16 +511,16 @@
         <v>user-student-1</v>
       </c>
       <c r="C3" t="str">
-        <v>7th</v>
+        <v>4th</v>
       </c>
       <c r="D3" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E3" t="str">
-        <v>ch-tam4-1</v>
+        <v>அன்னைத் தமிழே</v>
       </c>
       <c r="F3" t="str">
-        <v>அன்னைத் தமிழ் அரங்கம்</v>
+        <v>Tamil Chapter Quiz</v>
       </c>
       <c r="G3">
         <v>900</v>
@@ -549,28 +549,28 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Priya Sharma</v>
+        <v>Student Scholar</v>
       </c>
       <c r="B4" t="str">
-        <v>USER002</v>
+        <v>user-student-1</v>
       </c>
       <c r="C4" t="str">
         <v>7th</v>
       </c>
       <c r="D4" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E4" t="str">
-        <v>Chapter 2: Algebra Expressions</v>
+        <v>ch-tam4-1</v>
       </c>
       <c r="F4" t="str">
-        <v>Algebra Mastery Quiz</v>
+        <v>அன்னைத் தமிழ் அரங்கம்</v>
       </c>
       <c r="G4">
-        <v>95</v>
+        <v>900</v>
       </c>
       <c r="H4" t="str">
-        <v>95%</v>
+        <v>90%</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -582,10 +582,10 @@
         <v>1</v>
       </c>
       <c r="L4" t="str">
-        <v>04:40 mins</v>
+        <v>02:21 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>04-09-2026 23:14:28</v>
+        <v>05-09-2026 10:54:56</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -629,7 +629,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>04-09-2026 23:01:42</v>
+        <v>04-09-2026 23:14:28</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -673,7 +673,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>04-09-2026 22:19:16</v>
+        <v>04-09-2026 23:01:42</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -717,7 +717,7 @@
         <v>04:40 mins</v>
       </c>
       <c r="M7" t="str">
-        <v>04-09-2026 22:00:55</v>
+        <v>04-09-2026 22:19:16</v>
       </c>
       <c r="N7" t="str">
         <v>PASSED</v>
@@ -725,28 +725,28 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>John</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B8" t="str">
-        <v>USER001</v>
+        <v>USER002</v>
       </c>
       <c r="C8" t="str">
         <v>7th</v>
       </c>
       <c r="D8" t="str">
-        <v>Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E8" t="str">
-        <v>Chapter 1: Measurement &amp; Motion</v>
+        <v>Chapter 2: Algebra Expressions</v>
       </c>
       <c r="F8" t="str">
-        <v>Interactive Chapter Quiz</v>
+        <v>Algebra Mastery Quiz</v>
       </c>
       <c r="G8">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H8" t="str">
-        <v>90%</v>
+        <v>95%</v>
       </c>
       <c r="I8">
         <v>10</v>
@@ -758,10 +758,10 @@
         <v>1</v>
       </c>
       <c r="L8" t="str">
-        <v>05:30 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M8" t="str">
-        <v>04-09-2026 14:15:22</v>
+        <v>04-09-2026 22:00:55</v>
       </c>
       <c r="N8" t="str">
         <v>PASSED</v>
@@ -778,34 +778,34 @@
         <v>7th</v>
       </c>
       <c r="D9" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E9" t="str">
-        <v>Chapter 1: Number System: Integers</v>
+        <v>Chapter 1: Measurement &amp; Motion</v>
       </c>
       <c r="F9" t="str">
-        <v>Integer Operations Challenge</v>
+        <v>Interactive Chapter Quiz</v>
       </c>
       <c r="G9">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H9" t="str">
-        <v>80%</v>
+        <v>90%</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" t="str">
-        <v>06:15 mins</v>
+        <v>05:30 mins</v>
       </c>
       <c r="M9" t="str">
-        <v>04-09-2026 15:10:05</v>
+        <v>04-09-2026 14:15:22</v>
       </c>
       <c r="N9" t="str">
         <v>PASSED</v>
@@ -822,34 +822,34 @@
         <v>7th</v>
       </c>
       <c r="D10" t="str">
-        <v>English</v>
+        <v>Mathematics</v>
       </c>
       <c r="E10" t="str">
-        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
+        <v>Chapter 1: Number System: Integers</v>
       </c>
       <c r="F10" t="str">
-        <v>Grammar &amp; Vocabulary Quiz</v>
+        <v>Integer Operations Challenge</v>
       </c>
       <c r="G10">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H10" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I10">
         <v>10</v>
       </c>
       <c r="J10">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10" t="str">
-        <v>04:40 mins</v>
+        <v>06:15 mins</v>
       </c>
       <c r="M10" t="str">
-        <v>04-09-2026 15:45:18</v>
+        <v>04-09-2026 15:10:05</v>
       </c>
       <c r="N10" t="str">
         <v>PASSED</v>
@@ -857,22 +857,22 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Priya Sharma</v>
+        <v>John</v>
       </c>
       <c r="B11" t="str">
-        <v>USER002</v>
+        <v>USER001</v>
       </c>
       <c r="C11" t="str">
-        <v>8th</v>
+        <v>7th</v>
       </c>
       <c r="D11" t="str">
-        <v>Tamil</v>
+        <v>English</v>
       </c>
       <c r="E11" t="str">
-        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
+        <v>Chapter 1: Eidgah (Prose &amp; Grammar)</v>
       </c>
       <c r="F11" t="str">
-        <v>Tamil Literature Quiz</v>
+        <v>Grammar &amp; Vocabulary Quiz</v>
       </c>
       <c r="G11">
         <v>100</v>
@@ -890,10 +890,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="str">
-        <v>04:15 mins</v>
+        <v>04:40 mins</v>
       </c>
       <c r="M11" t="str">
-        <v>04-09-2026 11:20:45</v>
+        <v>04-09-2026 15:45:18</v>
       </c>
       <c r="N11" t="str">
         <v>PASSED</v>
@@ -910,34 +910,34 @@
         <v>8th</v>
       </c>
       <c r="D12" t="str">
-        <v>Science</v>
+        <v>Tamil</v>
       </c>
       <c r="E12" t="str">
-        <v>Chapter 1: Measurement</v>
+        <v>Chapter 1: தமிழ் இன்பம் (Tamil Inbam)</v>
       </c>
       <c r="F12" t="str">
-        <v>SI Unit &amp; Mechanics Quiz</v>
+        <v>Tamil Literature Quiz</v>
       </c>
       <c r="G12">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H12" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I12">
         <v>10</v>
       </c>
       <c r="J12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" t="str">
-        <v>05:05 mins</v>
+        <v>04:15 mins</v>
       </c>
       <c r="M12" t="str">
-        <v>04-09-2026 12:35:10</v>
+        <v>04-09-2026 11:20:45</v>
       </c>
       <c r="N12" t="str">
         <v>PASSED</v>
@@ -945,43 +945,43 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Arun Kumar</v>
+        <v>Priya Sharma</v>
       </c>
       <c r="B13" t="str">
-        <v>USER003</v>
+        <v>USER002</v>
       </c>
       <c r="C13" t="str">
-        <v>6th</v>
+        <v>8th</v>
       </c>
       <c r="D13" t="str">
         <v>Science</v>
       </c>
       <c r="E13" t="str">
-        <v>Chapter 1: Measurements &amp; Motion</v>
+        <v>Chapter 1: Measurement</v>
       </c>
       <c r="F13" t="str">
-        <v>Motion &amp; Scales Quest</v>
+        <v>SI Unit &amp; Mechanics Quiz</v>
       </c>
       <c r="G13">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H13" t="str">
-        <v>70%</v>
+        <v>90%</v>
       </c>
       <c r="I13">
         <v>10</v>
       </c>
       <c r="J13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L13" t="str">
-        <v>07:20 mins</v>
+        <v>05:05 mins</v>
       </c>
       <c r="M13" t="str">
-        <v>04-09-2026 09:30:12</v>
+        <v>04-09-2026 12:35:10</v>
       </c>
       <c r="N13" t="str">
         <v>PASSED</v>
@@ -998,37 +998,37 @@
         <v>6th</v>
       </c>
       <c r="D14" t="str">
-        <v>Mathematics</v>
+        <v>Science</v>
       </c>
       <c r="E14" t="str">
-        <v>Chapter 1: Numbers &amp; Operations</v>
+        <v>Chapter 1: Measurements &amp; Motion</v>
       </c>
       <c r="F14" t="str">
-        <v>Numbers Mastery Quiz</v>
+        <v>Motion &amp; Scales Quest</v>
       </c>
       <c r="G14">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H14" t="str">
-        <v>60%</v>
+        <v>70%</v>
       </c>
       <c r="I14">
         <v>10</v>
       </c>
       <c r="J14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14" t="str">
-        <v>08:15 mins</v>
+        <v>07:20 mins</v>
       </c>
       <c r="M14" t="str">
-        <v>04-09-2026 10:15:30</v>
+        <v>04-09-2026 09:30:12</v>
       </c>
       <c r="N14" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
     </row>
     <row r="15">
@@ -1048,72 +1048,72 @@
         <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F15" t="str">
-        <v>Numbers Mastery Quiz (Retry)</v>
+        <v>Numbers Mastery Quiz</v>
       </c>
       <c r="G15">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="H15" t="str">
-        <v>90%</v>
+        <v>60%</v>
       </c>
       <c r="I15">
         <v>10</v>
       </c>
       <c r="J15">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L15" t="str">
-        <v>05:45 mins</v>
+        <v>08:15 mins</v>
       </c>
       <c r="M15" t="str">
-        <v>04-09-2026 10:45:00</v>
+        <v>04-09-2026 10:15:30</v>
       </c>
       <c r="N15" t="str">
-        <v>PASSED</v>
+        <v>FAILED</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Divya Nair</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="B16" t="str">
-        <v>USER004</v>
+        <v>USER003</v>
       </c>
       <c r="C16" t="str">
-        <v>5th</v>
+        <v>6th</v>
       </c>
       <c r="D16" t="str">
-        <v>Social Science</v>
+        <v>Mathematics</v>
       </c>
       <c r="E16" t="str">
-        <v>Chapter 1: Introduction to Social Science</v>
+        <v>Chapter 1: Numbers &amp; Operations</v>
       </c>
       <c r="F16" t="str">
-        <v>Continents &amp; Oceans Quiz</v>
+        <v>Numbers Mastery Quiz (Retry)</v>
       </c>
       <c r="G16">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H16" t="str">
-        <v>100%</v>
+        <v>90%</v>
       </c>
       <c r="I16">
         <v>10</v>
       </c>
       <c r="J16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="str">
-        <v>03:50 mins</v>
+        <v>05:45 mins</v>
       </c>
       <c r="M16" t="str">
-        <v>04-09-2026 13:00:25</v>
+        <v>04-09-2026 10:45:00</v>
       </c>
       <c r="N16" t="str">
         <v>PASSED</v>
@@ -1121,22 +1121,22 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Student Scholar</v>
+        <v>Divya Nair</v>
       </c>
       <c r="B17" t="str">
-        <v>usr-student-1</v>
+        <v>USER004</v>
       </c>
       <c r="C17" t="str">
-        <v>4th</v>
+        <v>5th</v>
       </c>
       <c r="D17" t="str">
-        <v>Tamil</v>
+        <v>Social Science</v>
       </c>
       <c r="E17" t="str">
-        <v>Chapter 1: அன்னைத் தமிழே</v>
+        <v>Chapter 1: Introduction to Social Science</v>
       </c>
       <c r="F17" t="str">
-        <v>Tamil Poem &amp; Grammar Quiz</v>
+        <v>Continents &amp; Oceans Quiz</v>
       </c>
       <c r="G17">
         <v>100</v>
@@ -1154,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="L17" t="str">
-        <v>04:10 mins</v>
+        <v>03:50 mins</v>
       </c>
       <c r="M17" t="str">
-        <v>04-09-2026 14:00:15</v>
+        <v>04-09-2026 13:00:25</v>
       </c>
       <c r="N17" t="str">
         <v>PASSED</v>
@@ -1171,45 +1171,89 @@
         <v>usr-student-1</v>
       </c>
       <c r="C18" t="str">
-        <v>11th</v>
+        <v>4th</v>
       </c>
       <c r="D18" t="str">
-        <v>Chemistry</v>
+        <v>Tamil</v>
       </c>
       <c r="E18" t="str">
-        <v>Chapter 3: Periodic Classification</v>
+        <v>Chapter 1: அன்னைத் தமிழே</v>
       </c>
       <c r="F18" t="str">
-        <v>Grid Reconstruction Game</v>
+        <v>Tamil Poem &amp; Grammar Quiz</v>
       </c>
       <c r="G18">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="H18" t="str">
         <v>100%</v>
       </c>
       <c r="I18">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18" t="str">
+        <v>04:10 mins</v>
+      </c>
+      <c r="M18" t="str">
+        <v>04-09-2026 14:00:15</v>
+      </c>
+      <c r="N18" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B19" t="str">
+        <v>usr-student-1</v>
+      </c>
+      <c r="C19" t="str">
+        <v>11th</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Chapter 3: Periodic Classification</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Grid Reconstruction Game</v>
+      </c>
+      <c r="G19">
+        <v>150</v>
+      </c>
+      <c r="H19" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+      <c r="J19">
+        <v>3</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19" t="str">
         <v>03:20 mins</v>
       </c>
-      <c r="M18" t="str">
+      <c r="M19" t="str">
         <v>04-09-2026 15:30:00</v>
       </c>
-      <c r="N18" t="str">
+      <c r="N19" t="str">
         <v>COMPLETED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): update runtime data files after local testing session
- registered_users.json: updated user records (admin/teacher seeds + any newly registered students)
- user_activity_history.json: updated with real quiz activity records from local test runs
- user_game_progress.json: updated with offline fallback progress entries written during local testing
- EduNova_User_Activity_Report.xlsx: regenerated activity report reflecting latest quiz sessions
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -461,10 +461,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Sandy</v>
+        <v>San</v>
       </c>
       <c r="B2" t="str">
-        <v>usr-1788540894082-4sekc</v>
+        <v>usr-1788766211877-8z84d</v>
       </c>
       <c r="C2" t="str">
         <v>4th</v>
@@ -479,25 +479,25 @@
         <v>Tamil Chapter Quiz</v>
       </c>
       <c r="G2">
-        <v>900</v>
+        <v>800</v>
       </c>
       <c r="H2" t="str">
-        <v>90%</v>
+        <v>80%</v>
       </c>
       <c r="I2">
         <v>10</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" t="str">
-        <v>00:54 mins</v>
+        <v>00:50 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>05-09-2026 22:47:05</v>
+        <v>07-09-2026 13:03:18</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -508,7 +508,7 @@
         <v>Student Scholar</v>
       </c>
       <c r="B3" t="str">
-        <v>usr-1788540894082-4sekc</v>
+        <v>usr-1788766211877-8z84d</v>
       </c>
       <c r="C3" t="str">
         <v>7th</v>
@@ -523,33 +523,209 @@
         <v>அன்னைத் தமிழ் அரங்கம்</v>
       </c>
       <c r="G3">
-        <v>900</v>
+        <v>800</v>
       </c>
       <c r="H3" t="str">
-        <v>90%</v>
+        <v>80%</v>
       </c>
       <c r="I3">
         <v>10</v>
       </c>
       <c r="J3">
+        <v>8</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3" t="str">
+        <v>00:50 mins</v>
+      </c>
+      <c r="M3" t="str">
+        <v>07-09-2026 13:03:18</v>
+      </c>
+      <c r="N3" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>San</v>
+      </c>
+      <c r="B4" t="str">
+        <v>usr-1788766211877-8z84d</v>
+      </c>
+      <c r="C4" t="str">
+        <v>4th</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Tamil</v>
+      </c>
+      <c r="E4" t="str">
+        <v>அன்னைத் தமிழே</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Tamil Chapter Quiz</v>
+      </c>
+      <c r="G4">
+        <v>1000</v>
+      </c>
+      <c r="H4" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I4">
+        <v>10</v>
+      </c>
+      <c r="J4">
+        <v>10</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
+        <v>00:52 mins</v>
+      </c>
+      <c r="M4" t="str">
+        <v>07-09-2026 13:01:48</v>
+      </c>
+      <c r="N4" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B5" t="str">
+        <v>usr-1788766211877-8z84d</v>
+      </c>
+      <c r="C5" t="str">
+        <v>7th</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Science</v>
+      </c>
+      <c r="E5" t="str">
+        <v>ch-tam4-1</v>
+      </c>
+      <c r="F5" t="str">
+        <v>அன்னைத் தமிழ் அரங்கம்</v>
+      </c>
+      <c r="G5">
+        <v>1000</v>
+      </c>
+      <c r="H5" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>10</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v>00:52 mins</v>
+      </c>
+      <c r="M5" t="str">
+        <v>07-09-2026 13:01:48</v>
+      </c>
+      <c r="N5" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Sandy</v>
+      </c>
+      <c r="B6" t="str">
+        <v>usr-1788540894082-4sekc</v>
+      </c>
+      <c r="C6" t="str">
+        <v>4th</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Tamil</v>
+      </c>
+      <c r="E6" t="str">
+        <v>அன்னைத் தமிழே</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Tamil Chapter Quiz</v>
+      </c>
+      <c r="G6">
+        <v>900</v>
+      </c>
+      <c r="H6" t="str">
+        <v>90%</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
+      </c>
+      <c r="J6">
         <v>9</v>
       </c>
-      <c r="K3">
+      <c r="K6">
         <v>1</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L6" t="str">
         <v>00:54 mins</v>
       </c>
-      <c r="M3" t="str">
+      <c r="M6" t="str">
         <v>05-09-2026 22:47:05</v>
       </c>
-      <c r="N3" t="str">
+      <c r="N6" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B7" t="str">
+        <v>usr-1788540894082-4sekc</v>
+      </c>
+      <c r="C7" t="str">
+        <v>7th</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Science</v>
+      </c>
+      <c r="E7" t="str">
+        <v>ch-tam4-1</v>
+      </c>
+      <c r="F7" t="str">
+        <v>அன்னைத் தமிழ் அரங்கம்</v>
+      </c>
+      <c r="G7">
+        <v>900</v>
+      </c>
+      <c r="H7" t="str">
+        <v>90%</v>
+      </c>
+      <c r="I7">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>9</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="str">
+        <v>00:54 mins</v>
+      </c>
+      <c r="M7" t="str">
+        <v>05-09-2026 22:47:05</v>
+      </c>
+      <c r="N7" t="str">
         <v>PASSED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(theme): ensure full text and UI element visibility in light mode for teacher and admin modules
</commit_message>
<xml_diff>
--- a/backend/reports/EduNova_User_Activity_Report.xlsx
+++ b/backend/reports/EduNova_User_Activity_Report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N9"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -473,7 +473,7 @@
         <v>Tamil</v>
       </c>
       <c r="E2" t="str">
-        <v>அன்னைத் தமிழே</v>
+        <v>பனிமலைப் பயணம்</v>
       </c>
       <c r="F2" t="str">
         <v>Tamil Chapter Quiz</v>
@@ -494,10 +494,10 @@
         <v>2</v>
       </c>
       <c r="L2" t="str">
-        <v>00:50 mins</v>
+        <v>01:40 mins</v>
       </c>
       <c r="M2" t="str">
-        <v>07-09-2026 13:03:18</v>
+        <v>07-09-2026 13:25:43</v>
       </c>
       <c r="N2" t="str">
         <v>PASSED</v>
@@ -517,10 +517,10 @@
         <v>Science</v>
       </c>
       <c r="E3" t="str">
-        <v>ch-tam4-1</v>
+        <v>ch-tam4-2</v>
       </c>
       <c r="F3" t="str">
-        <v>அன்னைத் தமிழ் அரங்கம்</v>
+        <v>பனிமலை அரங்கம்</v>
       </c>
       <c r="G3">
         <v>800</v>
@@ -538,10 +538,10 @@
         <v>2</v>
       </c>
       <c r="L3" t="str">
-        <v>00:50 mins</v>
+        <v>01:40 mins</v>
       </c>
       <c r="M3" t="str">
-        <v>07-09-2026 13:03:18</v>
+        <v>07-09-2026 13:25:43</v>
       </c>
       <c r="N3" t="str">
         <v>PASSED</v>
@@ -567,25 +567,25 @@
         <v>Tamil Chapter Quiz</v>
       </c>
       <c r="G4">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="H4" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I4">
         <v>10</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L4" t="str">
-        <v>00:52 mins</v>
+        <v>00:50 mins</v>
       </c>
       <c r="M4" t="str">
-        <v>07-09-2026 13:01:48</v>
+        <v>07-09-2026 13:03:18</v>
       </c>
       <c r="N4" t="str">
         <v>PASSED</v>
@@ -611,25 +611,25 @@
         <v>அன்னைத் தமிழ் அரங்கம்</v>
       </c>
       <c r="G5">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="H5" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I5">
         <v>10</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L5" t="str">
-        <v>00:52 mins</v>
+        <v>00:50 mins</v>
       </c>
       <c r="M5" t="str">
-        <v>07-09-2026 13:01:48</v>
+        <v>07-09-2026 13:03:18</v>
       </c>
       <c r="N5" t="str">
         <v>PASSED</v>
@@ -637,10 +637,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sandy</v>
+        <v>San</v>
       </c>
       <c r="B6" t="str">
-        <v>usr-1788540894082-4sekc</v>
+        <v>usr-1788766211877-8z84d</v>
       </c>
       <c r="C6" t="str">
         <v>4th</v>
@@ -655,25 +655,25 @@
         <v>Tamil Chapter Quiz</v>
       </c>
       <c r="G6">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="H6" t="str">
-        <v>90%</v>
+        <v>100%</v>
       </c>
       <c r="I6">
         <v>10</v>
       </c>
       <c r="J6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" t="str">
-        <v>00:54 mins</v>
+        <v>00:52 mins</v>
       </c>
       <c r="M6" t="str">
-        <v>05-09-2026 22:47:05</v>
+        <v>07-09-2026 13:01:48</v>
       </c>
       <c r="N6" t="str">
         <v>PASSED</v>
@@ -684,7 +684,7 @@
         <v>Student Scholar</v>
       </c>
       <c r="B7" t="str">
-        <v>usr-1788540894082-4sekc</v>
+        <v>usr-1788766211877-8z84d</v>
       </c>
       <c r="C7" t="str">
         <v>7th</v>
@@ -699,33 +699,121 @@
         <v>அன்னைத் தமிழ் அரங்கம்</v>
       </c>
       <c r="G7">
+        <v>1000</v>
+      </c>
+      <c r="H7" t="str">
+        <v>100%</v>
+      </c>
+      <c r="I7">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>10</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="str">
+        <v>00:52 mins</v>
+      </c>
+      <c r="M7" t="str">
+        <v>07-09-2026 13:01:48</v>
+      </c>
+      <c r="N7" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Sandy</v>
+      </c>
+      <c r="B8" t="str">
+        <v>usr-1788540894082-4sekc</v>
+      </c>
+      <c r="C8" t="str">
+        <v>4th</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Tamil</v>
+      </c>
+      <c r="E8" t="str">
+        <v>அன்னைத் தமிழே</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Tamil Chapter Quiz</v>
+      </c>
+      <c r="G8">
         <v>900</v>
       </c>
-      <c r="H7" t="str">
+      <c r="H8" t="str">
         <v>90%</v>
       </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
+      <c r="I8">
+        <v>10</v>
+      </c>
+      <c r="J8">
         <v>9</v>
       </c>
-      <c r="K7">
+      <c r="K8">
         <v>1</v>
       </c>
-      <c r="L7" t="str">
+      <c r="L8" t="str">
         <v>00:54 mins</v>
       </c>
-      <c r="M7" t="str">
+      <c r="M8" t="str">
         <v>05-09-2026 22:47:05</v>
       </c>
-      <c r="N7" t="str">
+      <c r="N8" t="str">
+        <v>PASSED</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Student Scholar</v>
+      </c>
+      <c r="B9" t="str">
+        <v>usr-1788540894082-4sekc</v>
+      </c>
+      <c r="C9" t="str">
+        <v>7th</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Science</v>
+      </c>
+      <c r="E9" t="str">
+        <v>ch-tam4-1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>அன்னைத் தமிழ் அரங்கம்</v>
+      </c>
+      <c r="G9">
+        <v>900</v>
+      </c>
+      <c r="H9" t="str">
+        <v>90%</v>
+      </c>
+      <c r="I9">
+        <v>10</v>
+      </c>
+      <c r="J9">
+        <v>9</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9" t="str">
+        <v>00:54 mins</v>
+      </c>
+      <c r="M9" t="str">
+        <v>05-09-2026 22:47:05</v>
+      </c>
+      <c r="N9" t="str">
         <v>PASSED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>